<commit_message>
Ajustando estrutura de pastas
</commit_message>
<xml_diff>
--- a/archives/jira_cards.xlsx
+++ b/archives/jira_cards.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H109"/>
+  <dimension ref="A1:H108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -723,22 +723,22 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TENSYLON-674</t>
+          <t>MANTA-30807</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Tensylon</t>
+          <t>Manta</t>
         </is>
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/TENSYLON-674</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30807</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>30281</t>
+          <t>30439 PEDIDO AVULSO</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -749,11 +749,6 @@
       <c r="F8" t="inlineStr">
         <is>
           <t>🟢RECEBIDO LIBERADO</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>MERCEDES-BENZ - GLS SUV - 2026</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -765,7 +760,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MANTA-30807</t>
+          <t>MANTA-30781</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -775,29 +770,39 @@
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30807</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30781</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>30439 PEDIDO AVULSO</t>
+          <t>30911 PED AVULSO</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Liberado Engenharia</t>
+          <t>A Produzir</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
           <t>🟢RECEBIDO LIBERADO</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>VOLVO - XC90 - 2026</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>09/03/2026</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>MANTA-30781</t>
+          <t>MANTA-30763</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -807,34 +812,39 @@
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30781</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30763</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>30911 PED AVULSO</t>
+          <t>31136 - ALT</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>A Produzir</t>
+          <t>Liberado Engenharia</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>🟢RECEBIDO LIBERADO</t>
+          <t>⚪️RECEBIDO ENCAMINHADO</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>VOLVO - XC90 - 2026</t>
+          <t>TOYOTA - COROLLA SEDAN - 2026</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>13/03/2026</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MANTA-30763</t>
+          <t>MANTA-30740</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -844,12 +854,12 @@
       </c>
       <c r="C11" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30763</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30740</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>31136 - ALT</t>
+          <t>31140</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -876,7 +886,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MANTA-30740</t>
+          <t>MANTA-30739</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -886,12 +896,12 @@
       </c>
       <c r="C12" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30740</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30739</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>31140</t>
+          <t>31139</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -918,7 +928,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MANTA-30739</t>
+          <t>MANTA-30738</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -928,12 +938,12 @@
       </c>
       <c r="C13" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30739</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30738</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>31139</t>
+          <t>31138</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -960,7 +970,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MANTA-30738</t>
+          <t>MANTA-30737</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -970,12 +980,12 @@
       </c>
       <c r="C14" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30738</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30737</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>31138</t>
+          <t>31137</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1002,7 +1012,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>MANTA-30737</t>
+          <t>MANTA-30735</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1012,12 +1022,12 @@
       </c>
       <c r="C15" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30737</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30735</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>31137</t>
+          <t>31135</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1044,7 +1054,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MANTA-30735</t>
+          <t>MANTA-30734</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1054,17 +1064,17 @@
       </c>
       <c r="C16" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30735</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30734</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>31135</t>
+          <t>31134</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Liberado Engenharia</t>
+          <t>A Produzir</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1079,14 +1089,14 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>10/03/2026</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>MANTA-30734</t>
+          <t>MANTA-30733</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1096,17 +1106,17 @@
       </c>
       <c r="C17" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30734</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30733</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>31134</t>
+          <t>31133</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>A Produzir</t>
+          <t>Liberado Engenharia</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1121,14 +1131,14 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>13/03/2026</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>MANTA-30733</t>
+          <t>MANTA-30732</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1138,12 +1148,12 @@
       </c>
       <c r="C18" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30733</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30732</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>31133</t>
+          <t>31132</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1158,7 +1168,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA SEDAN - 2026</t>
+          <t>TOYOTA - COROLLA CROSS - 2026</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1170,7 +1180,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>MANTA-30732</t>
+          <t>MANTA-30730</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1180,12 +1190,12 @@
       </c>
       <c r="C19" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30732</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30730</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>31132</t>
+          <t>31130</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1212,7 +1222,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MANTA-30730</t>
+          <t>MANTA-30720</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1222,12 +1232,12 @@
       </c>
       <c r="C20" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30730</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30720</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>31130</t>
+          <t>30931 - ALT</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1237,7 +1247,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>⚪️RECEBIDO ENCAMINHADO</t>
+          <t>🟢RECEBIDO LIBERADO</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1254,7 +1264,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MANTA-30720</t>
+          <t>MANTA-30718</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1264,12 +1274,12 @@
       </c>
       <c r="C21" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30720</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30718</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>30931 - ALT</t>
+          <t>31120</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1279,7 +1289,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>🟢RECEBIDO LIBERADO</t>
+          <t>⚪️RECEBIDO ENCAMINHADO</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1296,7 +1306,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>MANTA-30718</t>
+          <t>MANTA-30658</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1306,12 +1316,12 @@
       </c>
       <c r="C22" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30718</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30658</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>31120</t>
+          <t>31061</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1338,7 +1348,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MANTA-30658</t>
+          <t>MANTA-30657</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1348,12 +1358,12 @@
       </c>
       <c r="C23" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30658</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30657</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>31061</t>
+          <t>31060</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1380,7 +1390,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>MANTA-30657</t>
+          <t>MANTA-30656</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1390,12 +1400,12 @@
       </c>
       <c r="C24" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30657</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30656</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>31060</t>
+          <t>31059</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1422,7 +1432,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MANTA-30656</t>
+          <t>MANTA-30649</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1432,12 +1442,12 @@
       </c>
       <c r="C25" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30656</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30649</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>31059</t>
+          <t>31054</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1452,7 +1462,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA CROSS - 2026</t>
+          <t>TOYOTA - COROLLA SEDAN - 2026</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1464,7 +1474,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>MANTA-30649</t>
+          <t>MANTA-30647</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1474,12 +1484,12 @@
       </c>
       <c r="C26" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30649</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30647</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>31054</t>
+          <t>31052</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1494,19 +1504,19 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA SEDAN - 2026</t>
+          <t>JEEP - COMPASS SUV - 2026</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>10/03/2026</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>MANTA-30647</t>
+          <t>MANTA-30638</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1516,12 +1526,12 @@
       </c>
       <c r="C27" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30647</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30638</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>31052</t>
+          <t>31043</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1536,7 +1546,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>JEEP - COMPASS SUV - 2026</t>
+          <t>GWM - HAVAL H6 PHEV 19 - 2026</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1548,7 +1558,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>MANTA-30638</t>
+          <t>MANTA-30630</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1558,12 +1568,12 @@
       </c>
       <c r="C28" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30638</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30630</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>31043</t>
+          <t>31036</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1578,7 +1588,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>GWM - HAVAL H6 PHEV 19 - 2026</t>
+          <t>GWM - HAVAL H6 GT - 2026</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1590,7 +1600,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>MANTA-30630</t>
+          <t>MANTA-30628</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1600,12 +1610,12 @@
       </c>
       <c r="C29" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30630</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30628</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>31036</t>
+          <t>31034</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1620,7 +1630,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>GWM - HAVAL H6 GT - 2026</t>
+          <t>GWM - HAVAL H9 SUV - 2026</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1632,7 +1642,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>MANTA-30628</t>
+          <t>MANTA-30624</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1642,12 +1652,12 @@
       </c>
       <c r="C30" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30628</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30624</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>31034</t>
+          <t>31030</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1662,19 +1672,19 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>GWM - HAVAL H9 SUV - 2026</t>
+          <t>TOYOTA - COROLLA SEDAN - 2026</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>13/03/2026</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>MANTA-30624</t>
+          <t>MANTA-30622</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1684,12 +1694,12 @@
       </c>
       <c r="C31" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30624</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30622</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>31030</t>
+          <t>31028</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1699,7 +1709,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>⚪️RECEBIDO ENCAMINHADO</t>
+          <t>🟢RECEBIDO LIBERADO</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1716,7 +1726,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>MANTA-30622</t>
+          <t>MANTA-30619</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1726,12 +1736,12 @@
       </c>
       <c r="C32" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30622</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30619</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>31028</t>
+          <t>31025</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1741,7 +1751,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>🟢RECEBIDO LIBERADO</t>
+          <t>⚪️RECEBIDO ENCAMINHADO</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1758,7 +1768,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>MANTA-30619</t>
+          <t>MANTA-30615</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1768,12 +1778,12 @@
       </c>
       <c r="C33" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30619</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30615</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>31025</t>
+          <t>31021</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1783,12 +1793,12 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>⚪️RECEBIDO ENCAMINHADO</t>
+          <t>🟢RECEBIDO LIBERADO</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA SEDAN - 2026</t>
+          <t>TOYOTA - COROLLA CROSS - 2026</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -1800,7 +1810,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>MANTA-30615</t>
+          <t>MANTA-30613</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1810,12 +1820,12 @@
       </c>
       <c r="C34" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30615</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30613</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>31021</t>
+          <t>31019</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1842,7 +1852,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>MANTA-30613</t>
+          <t>MANTA-30610</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1852,12 +1862,12 @@
       </c>
       <c r="C35" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30613</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30610</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>31019</t>
+          <t>31016</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1867,7 +1877,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>🟢RECEBIDO LIBERADO</t>
+          <t>⚪️RECEBIDO ENCAMINHADO</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1884,7 +1894,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>MANTA-30610</t>
+          <t>MANTA-30609</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1894,12 +1904,12 @@
       </c>
       <c r="C36" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30610</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30609</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>31016</t>
+          <t>31015</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1909,7 +1919,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>⚪️RECEBIDO ENCAMINHADO</t>
+          <t>🟢RECEBIDO LIBERADO</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1926,7 +1936,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>MANTA-30609</t>
+          <t>MANTA-30608</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1936,12 +1946,12 @@
       </c>
       <c r="C37" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30609</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30608</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>31015</t>
+          <t>31014</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1968,7 +1978,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>MANTA-30608</t>
+          <t>MANTA-30607</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1978,12 +1988,12 @@
       </c>
       <c r="C38" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30608</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30607</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>31014</t>
+          <t>31013</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1998,7 +2008,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA CROSS - 2026</t>
+          <t>TOYOTA - COROLLA SEDAN - 2026</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2010,7 +2020,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>MANTA-30607</t>
+          <t>MANTA-30606</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2020,12 +2030,12 @@
       </c>
       <c r="C39" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30607</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30606</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>31013</t>
+          <t>31012</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2040,7 +2050,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA SEDAN - 2026</t>
+          <t>TOYOTA - COROLLA CROSS - 2026</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -2052,7 +2062,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>MANTA-30606</t>
+          <t>MANTA-30602</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2062,12 +2072,12 @@
       </c>
       <c r="C40" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30606</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30602</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>31012</t>
+          <t>31009</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2094,7 +2104,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>MANTA-30602</t>
+          <t>MANTA-30600</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2104,12 +2114,12 @@
       </c>
       <c r="C41" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30602</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30600</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>31009</t>
+          <t>31006</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2136,7 +2146,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>MANTA-30600</t>
+          <t>MANTA-30597</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2146,12 +2156,12 @@
       </c>
       <c r="C42" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30600</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30597</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>31006</t>
+          <t>31003</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2178,7 +2188,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>MANTA-30597</t>
+          <t>MANTA-30595</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2188,12 +2198,12 @@
       </c>
       <c r="C43" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30597</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30595</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>31003</t>
+          <t>31001</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2208,7 +2218,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA CROSS - 2026</t>
+          <t>TOYOTA - COROLLA SEDAN - 2026</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -2220,7 +2230,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>MANTA-30595</t>
+          <t>MANTA-30594</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2230,12 +2240,12 @@
       </c>
       <c r="C44" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30595</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30594</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>31001</t>
+          <t>31000</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2245,7 +2255,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>🟢RECEBIDO LIBERADO</t>
+          <t>⚪️RECEBIDO ENCAMINHADO</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2262,7 +2272,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>MANTA-30594</t>
+          <t>MANTA-30593</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2272,12 +2282,12 @@
       </c>
       <c r="C45" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30594</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30593</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>31000</t>
+          <t>30999</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2287,7 +2297,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>⚪️RECEBIDO ENCAMINHADO</t>
+          <t>🟢RECEBIDO LIBERADO</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2304,7 +2314,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>MANTA-30593</t>
+          <t>MANTA-30590</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2314,12 +2324,12 @@
       </c>
       <c r="C46" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30593</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30590</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>30999</t>
+          <t>30996</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2329,7 +2339,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>🟢RECEBIDO LIBERADO</t>
+          <t>⚪️RECEBIDO ENCAMINHADO</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2346,7 +2356,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>MANTA-30590</t>
+          <t>MANTA-30589</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2356,12 +2366,12 @@
       </c>
       <c r="C47" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30590</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30589</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>30996</t>
+          <t>30995</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2371,12 +2381,12 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>⚪️RECEBIDO ENCAMINHADO</t>
+          <t>🟢RECEBIDO LIBERADO</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA SEDAN - 2026</t>
+          <t>TOYOTA - COROLLA CROSS - 2026</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2388,7 +2398,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>MANTA-30589</t>
+          <t>MANTA-30588</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2398,12 +2408,12 @@
       </c>
       <c r="C48" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30589</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30588</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>30995</t>
+          <t>30994</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2430,7 +2440,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>MANTA-30588</t>
+          <t>MANTA-30586</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2440,12 +2450,12 @@
       </c>
       <c r="C49" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30588</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30586</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>30994</t>
+          <t>30992</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2472,7 +2482,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>MANTA-30586</t>
+          <t>MANTA-30585</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2482,12 +2492,12 @@
       </c>
       <c r="C50" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30586</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30585</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>30992</t>
+          <t>30991</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2514,7 +2524,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>MANTA-30585</t>
+          <t>MANTA-30584</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2524,12 +2534,12 @@
       </c>
       <c r="C51" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30585</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30584</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>30991</t>
+          <t>30990</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2544,7 +2554,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA CROSS - 2026</t>
+          <t>TOYOTA - COROLLA SEDAN - 2026</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -2556,7 +2566,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>MANTA-30584</t>
+          <t>MANTA-30583</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2566,12 +2576,12 @@
       </c>
       <c r="C52" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30584</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30583</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>30990</t>
+          <t>30989</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2598,7 +2608,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>MANTA-30583</t>
+          <t>MANTA-30582</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2608,12 +2618,12 @@
       </c>
       <c r="C53" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30583</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30582</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>30989</t>
+          <t>30988</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2640,7 +2650,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>MANTA-30582</t>
+          <t>MANTA-30581</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2650,12 +2660,12 @@
       </c>
       <c r="C54" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30582</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30581</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>30988</t>
+          <t>30987</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2682,7 +2692,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>MANTA-30581</t>
+          <t>MANTA-30580</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2692,12 +2702,12 @@
       </c>
       <c r="C55" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30581</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30580</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>30987</t>
+          <t>30986</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2724,7 +2734,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>MANTA-30580</t>
+          <t>MANTA-30579</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2734,12 +2744,12 @@
       </c>
       <c r="C56" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30580</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30579</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>30986</t>
+          <t>30985</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2766,7 +2776,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>MANTA-30579</t>
+          <t>MANTA-30578</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2776,12 +2786,12 @@
       </c>
       <c r="C57" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30579</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30578</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>30985</t>
+          <t>30984</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2808,7 +2818,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>MANTA-30578</t>
+          <t>MANTA-30577</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2818,12 +2828,12 @@
       </c>
       <c r="C58" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30578</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30577</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>30984</t>
+          <t>30983</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2850,7 +2860,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>MANTA-30577</t>
+          <t>MANTA-30576</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2860,12 +2870,12 @@
       </c>
       <c r="C59" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30577</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30576</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>30983</t>
+          <t>30982</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2892,7 +2902,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>MANTA-30576</t>
+          <t>MANTA-30575</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2902,12 +2912,12 @@
       </c>
       <c r="C60" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30576</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30575</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>30982</t>
+          <t>30981</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2934,7 +2944,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>MANTA-30575</t>
+          <t>MANTA-30574</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2944,12 +2954,12 @@
       </c>
       <c r="C61" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30575</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30574</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>30981</t>
+          <t>30980</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2964,7 +2974,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA SEDAN - 2026</t>
+          <t>TOYOTA - COROLLA CROSS - 2026</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -2976,7 +2986,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>MANTA-30574</t>
+          <t>MANTA-30573</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2986,12 +2996,12 @@
       </c>
       <c r="C62" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30574</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30573</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>30980</t>
+          <t>30979</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -3018,7 +3028,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>MANTA-30573</t>
+          <t>MANTA-30571</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3028,12 +3038,12 @@
       </c>
       <c r="C63" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30573</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30571</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>30979</t>
+          <t>30977</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -3048,7 +3058,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA CROSS - 2026</t>
+          <t>TOYOTA - COROLLA SEDAN - 2026</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -3060,7 +3070,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>MANTA-30571</t>
+          <t>MANTA-30570</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3070,12 +3080,12 @@
       </c>
       <c r="C64" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30571</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30570</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>30977</t>
+          <t>30976</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -3102,7 +3112,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>MANTA-30570</t>
+          <t>MANTA-30569</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3112,12 +3122,12 @@
       </c>
       <c r="C65" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30570</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30569</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>30976</t>
+          <t>30975</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -3144,7 +3154,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>MANTA-30569</t>
+          <t>MANTA-30568</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3154,12 +3164,12 @@
       </c>
       <c r="C66" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30569</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30568</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>30975</t>
+          <t>30974</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -3169,24 +3179,24 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>🟢RECEBIDO LIBERADO</t>
+          <t>⚪️RECEBIDO ENCAMINHADO</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA SEDAN - 2026</t>
+          <t>HONDA - WR-V - 2026</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>10/03/2026</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>MANTA-30568</t>
+          <t>MANTA-30567</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3196,12 +3206,12 @@
       </c>
       <c r="C67" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30568</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30567</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>30974</t>
+          <t>30973</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -3216,7 +3226,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>HONDA - WR-V - 2026</t>
+          <t>HONDA - NEW HR-V SUV - 2026</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -3228,7 +3238,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>MANTA-30567</t>
+          <t>MANTA-30542</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3238,12 +3248,12 @@
       </c>
       <c r="C68" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30567</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30542</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>30973</t>
+          <t>30948</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -3258,7 +3268,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>HONDA - NEW HR-V SUV - 2026</t>
+          <t>BMW - X3 SUV - 2026</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -3270,7 +3280,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>MANTA-30542</t>
+          <t>MANTA-30530</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3280,12 +3290,12 @@
       </c>
       <c r="C69" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30542</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30530</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>30948</t>
+          <t>30939</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -3300,19 +3310,19 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>BMW - X3 SUV - 2026</t>
+          <t>TOYOTA - COROLLA CROSS - 2026</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>13/03/2026</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>MANTA-30530</t>
+          <t>MANTA-30526</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3322,12 +3332,12 @@
       </c>
       <c r="C70" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30530</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30526</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>30939</t>
+          <t>30935</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -3337,24 +3347,24 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>⚪️RECEBIDO ENCAMINHADO</t>
+          <t>🟢RECEBIDO LIBERADO</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA CROSS - 2026</t>
+          <t>TOYOTA - COROLLA SEDAN - 2026</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>09/03/2026</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>MANTA-30526</t>
+          <t>MANTA-30525</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3364,12 +3374,12 @@
       </c>
       <c r="C71" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30526</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30525</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>30935</t>
+          <t>30934</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -3396,7 +3406,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>MANTA-30525</t>
+          <t>MANTA-30523</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3406,12 +3416,12 @@
       </c>
       <c r="C72" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30525</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30523</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>30934</t>
+          <t>30932</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -3438,7 +3448,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>MANTA-30523</t>
+          <t>MANTA-30521</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3448,12 +3458,12 @@
       </c>
       <c r="C73" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30523</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30521</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>30932</t>
+          <t>30930</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3468,19 +3478,19 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA SEDAN - 2026</t>
+          <t>TOYOTA - COROLLA CROSS - 2026</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>13/03/2026</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>MANTA-30521</t>
+          <t>MANTA-30515</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3490,12 +3500,12 @@
       </c>
       <c r="C74" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30521</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30515</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>30930</t>
+          <t>30924</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3522,7 +3532,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>MANTA-30515</t>
+          <t>MANTA-30514</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3532,12 +3542,12 @@
       </c>
       <c r="C75" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30515</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30514</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>30924</t>
+          <t>30923</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3564,7 +3574,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>MANTA-30514</t>
+          <t>MANTA-30513</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3574,12 +3584,12 @@
       </c>
       <c r="C76" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30514</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30513</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>30923</t>
+          <t>30922</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -3594,7 +3604,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA CROSS - 2026</t>
+          <t>TOYOTA - COROLLA SEDAN - 2026</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -3606,7 +3616,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>MANTA-30513</t>
+          <t>MANTA-30512</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3616,12 +3626,12 @@
       </c>
       <c r="C77" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30513</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30512</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>30922</t>
+          <t>30921</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -3648,7 +3658,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>MANTA-30512</t>
+          <t>MANTA-30511</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -3658,12 +3668,12 @@
       </c>
       <c r="C78" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30512</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30511</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>30921</t>
+          <t>30920</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -3690,7 +3700,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>MANTA-30511</t>
+          <t>MANTA-30510</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -3700,12 +3710,12 @@
       </c>
       <c r="C79" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30511</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30510</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>30920</t>
+          <t>30919</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -3720,7 +3730,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA SEDAN - 2026</t>
+          <t>TOYOTA - COROLLA CROSS - 2026</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -3732,7 +3742,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>MANTA-30510</t>
+          <t>MANTA-30509</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -3742,12 +3752,12 @@
       </c>
       <c r="C80" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30510</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30509</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>30919</t>
+          <t>30918</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -3757,7 +3767,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>🟢RECEBIDO LIBERADO</t>
+          <t>⚪️RECEBIDO ENCAMINHADO</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -3774,7 +3784,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>MANTA-30509</t>
+          <t>MANTA-30507</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -3784,12 +3794,12 @@
       </c>
       <c r="C81" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30509</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30507</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>30918</t>
+          <t>30916</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -3799,7 +3809,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>⚪️RECEBIDO ENCAMINHADO</t>
+          <t>🟢RECEBIDO LIBERADO</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -3816,7 +3826,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>MANTA-30507</t>
+          <t>MANTA-30506</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -3826,12 +3836,12 @@
       </c>
       <c r="C82" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30507</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30506</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>30916</t>
+          <t>30915</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -3851,14 +3861,14 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>10/03/2026</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>MANTA-30506</t>
+          <t>MANTA-30505</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -3868,12 +3878,12 @@
       </c>
       <c r="C83" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30506</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30505</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>30915</t>
+          <t>30914</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -3893,14 +3903,14 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>13/03/2026</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>MANTA-30505</t>
+          <t>MANTA-30504</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -3910,12 +3920,12 @@
       </c>
       <c r="C84" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30505</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30504</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>30914</t>
+          <t>30913</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -3925,24 +3935,24 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>🟢RECEBIDO LIBERADO</t>
+          <t>⚪️RECEBIDO ENCAMINHADO</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA CROSS - 2026</t>
+          <t>JAECOO - JAECOO 7 SUV - 2026</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>10/03/2026</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>MANTA-30504</t>
+          <t>MANTA-30479</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -3952,12 +3962,12 @@
       </c>
       <c r="C85" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30504</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30479</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>30913</t>
+          <t>30892</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -3972,7 +3982,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>JAECOO - JAECOO 7 SUV - 2026</t>
+          <t>LEXUS - NX 350 H SUV - 2026</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -3984,7 +3994,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>MANTA-30479</t>
+          <t>MANTA-30469</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -3994,12 +4004,12 @@
       </c>
       <c r="C86" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30479</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30469</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>30892</t>
+          <t>30882</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -4014,7 +4024,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>LEXUS - NX 350 H SUV - 2026</t>
+          <t>MINI - COOPER 04 PORTAS HATCH - 2026</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -4026,7 +4036,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>MANTA-30469</t>
+          <t>MANTA-30464</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4036,12 +4046,12 @@
       </c>
       <c r="C87" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30469</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30464</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>30882</t>
+          <t>30877</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4051,12 +4061,12 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>⚪️RECEBIDO ENCAMINHADO</t>
+          <t>🟢RECEBIDO LIBERADO</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>MINI - COOPER 04 PORTAS HATCH - 2026</t>
+          <t>TOYOTA - COROLLA CROSS - 2026</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -4068,7 +4078,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>MANTA-30464</t>
+          <t>MANTA-30463</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -4078,12 +4088,12 @@
       </c>
       <c r="C88" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30464</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30463</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>30877</t>
+          <t>30876</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -4098,19 +4108,19 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA CROSS - 2026</t>
+          <t>TOYOTA - COROLLA SEDAN - 2026</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>13/03/2026</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>MANTA-30463</t>
+          <t>MANTA-30462</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4120,12 +4130,12 @@
       </c>
       <c r="C89" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30463</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30462</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>30876</t>
+          <t>30875</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -4140,19 +4150,19 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA SEDAN - 2026</t>
+          <t>TOYOTA - COROLLA CROSS - 2026</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>10/03/2026</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>MANTA-30462</t>
+          <t>MANTA-30452</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -4162,12 +4172,12 @@
       </c>
       <c r="C90" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30462</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30452</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>30875</t>
+          <t>30865</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -4177,7 +4187,7 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>🟢RECEBIDO LIBERADO</t>
+          <t>⚪️RECEBIDO ENCAMINHADO</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -4187,14 +4197,14 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>13/03/2026</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>MANTA-30452</t>
+          <t>MANTA-30451</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4204,12 +4214,12 @@
       </c>
       <c r="C91" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30452</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30451</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>30865</t>
+          <t>30864</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -4224,19 +4234,19 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA CROSS - 2026</t>
+          <t>KIA - CARNIVAL VAN - 2025</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>10/03/2026</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>MANTA-30451</t>
+          <t>MANTA-30428</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -4246,12 +4256,12 @@
       </c>
       <c r="C92" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30451</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30428</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>30864</t>
+          <t>30841</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -4261,24 +4271,24 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>⚪️RECEBIDO ENCAMINHADO</t>
+          <t>🟢RECEBIDO LIBERADO</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>KIA - CARNIVAL VAN - 2025</t>
+          <t>TOYOTA - COROLLA SEDAN - 2026</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>13/03/2026</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>MANTA-30428</t>
+          <t>MANTA-30421</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -4288,12 +4298,12 @@
       </c>
       <c r="C93" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30428</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30421</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>30841</t>
+          <t>30834</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -4320,7 +4330,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>MANTA-30421</t>
+          <t>MANTA-30420</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -4330,12 +4340,12 @@
       </c>
       <c r="C94" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30421</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30420</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>30834</t>
+          <t>30833</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -4355,14 +4365,14 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>09/03/2026</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>MANTA-30420</t>
+          <t>MANTA-30367</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -4372,12 +4382,12 @@
       </c>
       <c r="C95" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30420</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30367</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>30833</t>
+          <t>30786</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4397,14 +4407,14 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>13/03/2026</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>MANTA-30367</t>
+          <t>MANTA-30309</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -4414,12 +4424,12 @@
       </c>
       <c r="C96" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30367</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30309</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>30786</t>
+          <t>30735</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -4434,19 +4444,19 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA SEDAN - 2026</t>
+          <t>TOYOTA - SW4 SUV - 2026</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>09/03/2026</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>MANTA-30309</t>
+          <t>MANTA-30257</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4456,12 +4466,12 @@
       </c>
       <c r="C97" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30309</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30257</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>30735</t>
+          <t>30687</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -4471,7 +4481,7 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>🟢RECEBIDO LIBERADO</t>
+          <t>⚪️RECEBIDO ENCAMINHADO</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -4481,14 +4491,14 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>13/03/2026</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>MANTA-30257</t>
+          <t>MANTA-30242</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -4498,12 +4508,12 @@
       </c>
       <c r="C98" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30257</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30242</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>30687</t>
+          <t>30674</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -4513,24 +4523,24 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>⚪️RECEBIDO ENCAMINHADO</t>
+          <t>🟢RECEBIDO LIBERADO</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>TOYOTA - SW4 SUV - 2026</t>
+          <t>TOYOTA - COROLLA CROSS - 2026</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>09/03/2026</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>MANTA-30242</t>
+          <t>MANTA-30224</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -4540,12 +4550,12 @@
       </c>
       <c r="C99" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30242</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30224</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>30674</t>
+          <t>30657</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -4555,24 +4565,24 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>🟢RECEBIDO LIBERADO</t>
+          <t>⚪️RECEBIDO ENCAMINHADO</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA CROSS - 2026</t>
+          <t>TOYOTA - SW4 SUV - 2026</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>13/03/2026</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>MANTA-30224</t>
+          <t>MANTA-30196</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -4582,12 +4592,12 @@
       </c>
       <c r="C100" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30224</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30196</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>30657</t>
+          <t>30632</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -4597,24 +4607,24 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>⚪️RECEBIDO ENCAMINHADO</t>
+          <t>🟢RECEBIDO LIBERADO</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>TOYOTA - SW4 SUV - 2026</t>
+          <t>TOYOTA - COROLLA SEDAN - 2026</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>09/03/2026</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>MANTA-30196</t>
+          <t>MANTA-30191</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -4624,12 +4634,12 @@
       </c>
       <c r="C101" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30196</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30191</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>30632</t>
+          <t>30628</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -4639,24 +4649,24 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>🟢RECEBIDO LIBERADO</t>
+          <t>⚪️RECEBIDO ENCAMINHADO</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA SEDAN - 2026</t>
+          <t>BMW - X3 SUV - 2026</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>10/03/2026</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>MANTA-30191</t>
+          <t>MANTA-30026</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -4666,12 +4676,12 @@
       </c>
       <c r="C102" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30191</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-30026</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>30628</t>
+          <t>30483</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -4686,7 +4696,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>BMW - X3 SUV - 2026</t>
+          <t>JEEP - COMMANDER SUV - 2026</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
@@ -4698,7 +4708,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>MANTA-30026</t>
+          <t>MANTA-29945</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -4708,12 +4718,12 @@
       </c>
       <c r="C103" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-30026</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-29945</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>30483</t>
+          <t>30412</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -4728,7 +4738,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>JEEP - COMMANDER SUV - 2026</t>
+          <t>GWM - HAVAL H6 HEV 2 - 2026</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
@@ -4740,7 +4750,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>MANTA-29945</t>
+          <t>MANTA-29923</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -4750,12 +4760,12 @@
       </c>
       <c r="C104" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-29945</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-29923</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>30412</t>
+          <t>30392</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -4765,24 +4775,24 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>⚪️RECEBIDO ENCAMINHADO</t>
+          <t>🟢RECEBIDO LIBERADO</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>GWM - HAVAL H6 HEV 2 - 2026</t>
+          <t>TOYOTA - COROLLA SEDAN - 2026</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>13/03/2026</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>MANTA-29923</t>
+          <t>MANTA-29866</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -4792,12 +4802,12 @@
       </c>
       <c r="C105" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-29923</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-29866</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>30392</t>
+          <t>30344</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -4807,12 +4817,12 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>🟢RECEBIDO LIBERADO</t>
+          <t>⚪️RECEBIDO ENCAMINHADO</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA SEDAN - 2026</t>
+          <t>LAND ROVER - DISCOVERY METROPOLITAN - 2024</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
@@ -4824,7 +4834,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>MANTA-29866</t>
+          <t>MANTA-29791</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -4834,12 +4844,12 @@
       </c>
       <c r="C106" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-29866</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-29791</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>30344</t>
+          <t>30281</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -4849,24 +4859,24 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>⚪️RECEBIDO ENCAMINHADO</t>
+          <t>🟢RECEBIDO LIBERADO</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>LAND ROVER - DISCOVERY METROPOLITAN - 2024</t>
+          <t>MERCEDES-BENZ - GLS SUV - 2026</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>13/03/2026</t>
+          <t>10/03/2026</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>MANTA-29791</t>
+          <t>MANTA-29372</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -4876,12 +4886,12 @@
       </c>
       <c r="C107" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-29791</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-29372</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>30281</t>
+          <t>29901</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -4896,19 +4906,19 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>MERCEDES-BENZ - GLS SUV - 2026</t>
+          <t>TOYOTA - COROLLA SEDAN - 2026</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>13/03/2026</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>MANTA-29372</t>
+          <t>MANTA-27100</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -4918,12 +4928,12 @@
       </c>
       <c r="C108" s="1" t="inlineStr">
         <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-29372</t>
+          <t>https://carboncars.atlassian.net/browse/MANTA-27100</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>29901</t>
+          <t>28192</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -4933,57 +4943,15 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>🟢RECEBIDO LIBERADO</t>
+          <t>⚪️RECEBIDO ENCAMINHADO</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>TOYOTA - COROLLA SEDAN - 2026</t>
+          <t>LEXUS - RX 500H SUV - 2025</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
-        <is>
-          <t>13/03/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="inlineStr">
-        <is>
-          <t>MANTA-27100</t>
-        </is>
-      </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>Manta</t>
-        </is>
-      </c>
-      <c r="C109" s="1" t="inlineStr">
-        <is>
-          <t>https://carboncars.atlassian.net/browse/MANTA-27100</t>
-        </is>
-      </c>
-      <c r="D109" t="inlineStr">
-        <is>
-          <t>28192</t>
-        </is>
-      </c>
-      <c r="E109" t="inlineStr">
-        <is>
-          <t>Liberado Engenharia</t>
-        </is>
-      </c>
-      <c r="F109" t="inlineStr">
-        <is>
-          <t>⚪️RECEBIDO ENCAMINHADO</t>
-        </is>
-      </c>
-      <c r="G109" t="inlineStr">
-        <is>
-          <t>LEXUS - RX 500H SUV - 2025</t>
-        </is>
-      </c>
-      <c r="H109" t="inlineStr">
         <is>
           <t>10/03/2026</t>
         </is>
@@ -5098,7 +5066,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C106" r:id="rId105"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C107" r:id="rId106"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C108" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C109" r:id="rId108"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>